<commit_message>
Cambios desde la compu de trabajo
</commit_message>
<xml_diff>
--- a/storage/CONTROL DE GEOS Y SABANAS.xlsx
+++ b/storage/CONTROL DE GEOS Y SABANAS.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P12"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str">
@@ -450,9 +450,559 @@
         <v>Ubicación Archivo</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2282439103</v>
+      </c>
+      <c r="C2" t="str">
+        <v>+522282439103</v>
+      </c>
+      <c r="D2" t="str">
+        <v>20/03/2026, 12:21</v>
+      </c>
+      <c r="E2" t="str">
+        <v>MTRE. HERRERA</v>
+      </c>
+      <c r="F2" t="str">
+        <v>AT&amp;T</v>
+      </c>
+      <c r="G2" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H2" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I2" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J2">
+        <v>19.5334</v>
+      </c>
+      <c r="K2">
+        <v>-96.9162</v>
+      </c>
+      <c r="L2">
+        <v>19.5334</v>
+      </c>
+      <c r="M2">
+        <v>-96.9162</v>
+      </c>
+      <c r="N2">
+        <v>250</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\522282439103\GEOLOCALIZACIONES\20-03-2026,\522282439103_POSITIVO_COCEFI.pdf</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2288576290</v>
+      </c>
+      <c r="C3" t="str">
+        <v>+522288576290</v>
+      </c>
+      <c r="D3" t="str">
+        <v>20/03/2026, 11:59</v>
+      </c>
+      <c r="E3" t="str">
+        <v>MTRE. HERRERA</v>
+      </c>
+      <c r="F3" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G3" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H3" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I3" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J3">
+        <v>19.4988</v>
+      </c>
+      <c r="K3">
+        <v>-96.8319</v>
+      </c>
+      <c r="L3">
+        <v>19.4988</v>
+      </c>
+      <c r="M3">
+        <v>-96.8319</v>
+      </c>
+      <c r="N3">
+        <v>1234</v>
+      </c>
+      <c r="O3" t="str">
+        <v>{"lat":19.4988,"lng":-96.8319,"azimuth":120,"range":1234,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P3" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\522288576290\GEOLOCALIZACIONES\20-03-2026,\522288576290_POSITIVA_COCEFI.pdf</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2291521507</v>
+      </c>
+      <c r="C4" t="str">
+        <v>+522291521507</v>
+      </c>
+      <c r="D4" t="str">
+        <v>20/03/2026, 12:01</v>
+      </c>
+      <c r="E4" t="str">
+        <v>MTRE. HERRERA</v>
+      </c>
+      <c r="F4" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G4" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H4" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I4" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J4">
+        <v>19.0944</v>
+      </c>
+      <c r="K4">
+        <v>-98.2072</v>
+      </c>
+      <c r="L4">
+        <v>19.0944</v>
+      </c>
+      <c r="M4">
+        <v>-98.2072</v>
+      </c>
+      <c r="N4">
+        <v>835</v>
+      </c>
+      <c r="O4" t="str">
+        <v>{"lat":19.0944,"lng":-98.2072,"azimuth":240,"range":835,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P4" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\522291521507\GEOLOCALIZACIONES\20-03-2026,\522291521507_POSITIVA_COCEFI.pdf</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2291587075</v>
+      </c>
+      <c r="C5" t="str">
+        <v>+522291587075</v>
+      </c>
+      <c r="D5" t="str">
+        <v>20/03/2026, 12:03</v>
+      </c>
+      <c r="E5" t="str">
+        <v>MTRE. HERRERA</v>
+      </c>
+      <c r="F5" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G5" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H5" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I5" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J5">
+        <v>18.7701</v>
+      </c>
+      <c r="K5">
+        <v>-95.7615</v>
+      </c>
+      <c r="L5">
+        <v>18.7701</v>
+      </c>
+      <c r="M5">
+        <v>-95.7615</v>
+      </c>
+      <c r="N5">
+        <v>1720</v>
+      </c>
+      <c r="O5" t="str">
+        <v>{"lat":18.7701,"lng":-95.7615,"azimuth":0,"range":1720,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P5" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\522291587075\GEOLOCALIZACIONES\20-03-2026,\522291587075_POSITIVA_COCEFI.pdf</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2299407081</v>
+      </c>
+      <c r="C6" t="str">
+        <v>+522299407081</v>
+      </c>
+      <c r="D6" t="str">
+        <v>20/03/2026, 11:55</v>
+      </c>
+      <c r="E6" t="str">
+        <v>MTRE. HERRERA</v>
+      </c>
+      <c r="F6" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G6" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H6" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I6" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J6">
+        <v>19.1126</v>
+      </c>
+      <c r="K6">
+        <v>-98.2778</v>
+      </c>
+      <c r="L6">
+        <v>19.1126</v>
+      </c>
+      <c r="M6">
+        <v>-98.2778</v>
+      </c>
+      <c r="N6">
+        <v>854</v>
+      </c>
+      <c r="O6" t="str">
+        <v>{"lat":19.1126,"lng":-98.2778,"azimuth":240,"range":854,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P6" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\522299407081\GEOLOCALIZACIONES\20-03-2026,\522299407081_POSITIVA_COCEFI.pdf</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>7333308709</v>
+      </c>
+      <c r="C7" t="str">
+        <v>+527333308709</v>
+      </c>
+      <c r="D7" t="str">
+        <v>20/03/2026, 10:17</v>
+      </c>
+      <c r="E7" t="str">
+        <v>MTRE. HERRERA</v>
+      </c>
+      <c r="F7" t="str">
+        <v>ALTAN</v>
+      </c>
+      <c r="G7" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H7" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I7" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J7">
+        <v>19.4149</v>
+      </c>
+      <c r="K7">
+        <v>-98.1188</v>
+      </c>
+      <c r="L7">
+        <v>19.4149</v>
+      </c>
+      <c r="M7">
+        <v>-98.1188</v>
+      </c>
+      <c r="N7">
+        <v>963</v>
+      </c>
+      <c r="O7" t="str">
+        <v>{"lat":19.4149,"lng":-98.1188,"azimuth":240,"range":963,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P7" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\527333308709\GEOLOCALIZACIONES\20-03-2026,\527333308709_POSITIVO-SO.pdf</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>9211155959</v>
+      </c>
+      <c r="C8" t="str">
+        <v>+529211155959</v>
+      </c>
+      <c r="D8" t="str">
+        <v>20/03/2026, 12:00</v>
+      </c>
+      <c r="E8" t="str">
+        <v>TTE ABARCA</v>
+      </c>
+      <c r="F8" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G8" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H8" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I8" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J8">
+        <v>18.1256</v>
+      </c>
+      <c r="K8">
+        <v>-94.4548</v>
+      </c>
+      <c r="L8">
+        <v>18.1256</v>
+      </c>
+      <c r="M8">
+        <v>-94.4548</v>
+      </c>
+      <c r="N8">
+        <v>1684</v>
+      </c>
+      <c r="O8" t="str">
+        <v>{"lat":18.1256,"lng":-94.4548,"azimuth":240,"range":1684,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P8" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\529211155959\GEOLOCALIZACIONES\20-03-2026,\529211155959_POSITIVA_COCEFI.pdf</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>9381566125</v>
+      </c>
+      <c r="C9" t="str">
+        <v>+529381566125</v>
+      </c>
+      <c r="D9" t="str">
+        <v>20/03/2026, 10:47</v>
+      </c>
+      <c r="E9" t="str">
+        <v>MTRE MELCHOR</v>
+      </c>
+      <c r="F9" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G9" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H9" t="str">
+        <v>COCEFI</v>
+      </c>
+      <c r="I9" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J9">
+        <v>18.6458</v>
+      </c>
+      <c r="K9">
+        <v>-91.8064</v>
+      </c>
+      <c r="L9">
+        <v>18.6458</v>
+      </c>
+      <c r="M9">
+        <v>-91.8064</v>
+      </c>
+      <c r="N9">
+        <v>1297</v>
+      </c>
+      <c r="O9" t="str">
+        <v>{"lat":18.6458,"lng":-91.8064,"azimuth":0,"range":1297,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P9" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\529381566125\GEOLOCALIZACIONES\20-03-2026,\529381566125_POSITIVO_CEREGINA-3.pdf</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>9381566125</v>
+      </c>
+      <c r="C10" t="str">
+        <v>+529381566125</v>
+      </c>
+      <c r="D10" t="str">
+        <v>20/03/2026, 16:16</v>
+      </c>
+      <c r="E10" t="str">
+        <v>CABO VELAZQUEZ</v>
+      </c>
+      <c r="F10" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G10" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H10" t="str">
+        <v>CEREGINA-3</v>
+      </c>
+      <c r="I10" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J10">
+        <v>18.6191</v>
+      </c>
+      <c r="K10">
+        <v>-92.2233</v>
+      </c>
+      <c r="L10">
+        <v>18.6191</v>
+      </c>
+      <c r="M10">
+        <v>-92.2233</v>
+      </c>
+      <c r="N10">
+        <v>896</v>
+      </c>
+      <c r="O10" t="str">
+        <v>{"lat":18.6191,"lng":-92.2233,"azimuth":0,"range":896,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P10" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\529381566125\GEOLOCALIZACIONES\20-03-2026,\529381566125_20032026_041708.pdf</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>9381566125</v>
+      </c>
+      <c r="C11" t="str">
+        <v>+529381566125</v>
+      </c>
+      <c r="D11" t="str">
+        <v>20/03/2026, 10:47</v>
+      </c>
+      <c r="E11" t="str">
+        <v>CABO VELAZQUEZ</v>
+      </c>
+      <c r="F11" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G11" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H11" t="str">
+        <v>CEREGINA-3</v>
+      </c>
+      <c r="I11" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J11">
+        <v>18.6458</v>
+      </c>
+      <c r="K11">
+        <v>-91.8064</v>
+      </c>
+      <c r="L11">
+        <v>18.6458</v>
+      </c>
+      <c r="M11">
+        <v>-91.8064</v>
+      </c>
+      <c r="N11">
+        <v>1297</v>
+      </c>
+      <c r="O11" t="str">
+        <v>{"lat":18.6458,"lng":-91.8064,"azimuth":0,"range":1297,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P11" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\529381566125\GEOLOCALIZACIONES\20-03-2026,\529381566125_POSITIVO_CEREGINA-3.pdf</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>4531506955</v>
+      </c>
+      <c r="C12" t="str">
+        <v>+524531506955</v>
+      </c>
+      <c r="D12" t="str">
+        <v>21/03/2026, 09:57</v>
+      </c>
+      <c r="E12" t="str">
+        <v>CABO VELAZQUEZ</v>
+      </c>
+      <c r="F12" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G12" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H12" t="str">
+        <v>LANCEROS</v>
+      </c>
+      <c r="I12" t="str">
+        <v>NEGATIVO</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12">
+        <v>400</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\524531506955\GEOLOCALIZACIONES\21-03-2026,\524531506955_21032026_095611.pdf</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add User registration flow, Prisma schema user model, and sync tracking documents
</commit_message>
<xml_diff>
--- a/storage/CONTROL DE GEOS Y SABANAS.xlsx
+++ b/storage/CONTROL DE GEOS Y SABANAS.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P15"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str">
@@ -1000,9 +1000,159 @@
         <v>C:\Users\DI-SO\Music\intellectus\project-intellectus\storage\524531506955\GEOLOCALIZACIONES\21-03-2026,\524531506955_21032026_095611.pdf</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>3221003735</v>
+      </c>
+      <c r="C13" t="str">
+        <v>+523221003735</v>
+      </c>
+      <c r="D13" t="str">
+        <v>10/02/2026, 11:38</v>
+      </c>
+      <c r="E13" t="str">
+        <v>CABO VELAZQUEZ</v>
+      </c>
+      <c r="F13" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G13" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H13" t="str">
+        <v>SO</v>
+      </c>
+      <c r="I13" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J13">
+        <v>20.6624</v>
+      </c>
+      <c r="K13">
+        <v>-103.3886</v>
+      </c>
+      <c r="L13">
+        <v>20.6624</v>
+      </c>
+      <c r="M13">
+        <v>-103.3886</v>
+      </c>
+      <c r="N13">
+        <v>800</v>
+      </c>
+      <c r="O13" t="str">
+        <v>{"lat":20.6624,"lng":-103.3886,"azimuth":120,"range":800,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P13" t="str">
+        <v>C:\Users\SO\Videos\intellectus\project-intellectus\storage\523221003735\GEOLOCALIZACIONES\10-02-2026,\523221003735 SECNAP POSITIVO.pdf</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>3221003735</v>
+      </c>
+      <c r="C14" t="str">
+        <v>+523221003735</v>
+      </c>
+      <c r="D14" t="str">
+        <v>10/02/2026, 14:07</v>
+      </c>
+      <c r="E14" t="str">
+        <v>CABO VELAZQUEZ</v>
+      </c>
+      <c r="F14" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G14" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H14" t="str">
+        <v>SO</v>
+      </c>
+      <c r="I14" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J14">
+        <v>20.721</v>
+      </c>
+      <c r="K14">
+        <v>-103.4156</v>
+      </c>
+      <c r="L14">
+        <v>20.721</v>
+      </c>
+      <c r="M14">
+        <v>-103.4156</v>
+      </c>
+      <c r="N14">
+        <v>756</v>
+      </c>
+      <c r="O14" t="str">
+        <v>{"lat":20.721,"lng":-103.4156,"azimuth":0,"range":756,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P14" t="str">
+        <v>C:\Users\SO\Videos\intellectus\project-intellectus\storage\523221003735\GEOLOCALIZACIONES\10-02-2026,\523221003735_ SECNAP_ POSITIVO_ C.pdf</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>3221049457</v>
+      </c>
+      <c r="C15" t="str">
+        <v>+523221049457</v>
+      </c>
+      <c r="D15" t="str">
+        <v>10/02/2026, 08:02</v>
+      </c>
+      <c r="E15" t="str">
+        <v>CABO GALICIA</v>
+      </c>
+      <c r="F15" t="str">
+        <v>TELCEL</v>
+      </c>
+      <c r="G15" t="str">
+        <v>GEO</v>
+      </c>
+      <c r="H15" t="str">
+        <v>SO</v>
+      </c>
+      <c r="I15" t="str">
+        <v>POSITIVO</v>
+      </c>
+      <c r="J15">
+        <v>21.4577</v>
+      </c>
+      <c r="K15">
+        <v>-104.9001</v>
+      </c>
+      <c r="L15">
+        <v>21.4577</v>
+      </c>
+      <c r="M15">
+        <v>-104.9001</v>
+      </c>
+      <c r="N15">
+        <v>400</v>
+      </c>
+      <c r="O15" t="str">
+        <v>{"lat":21.4577,"lng":-104.9001,"azimuth":120,"range":400,"widthDeg":120,"azimuthSource":"inferred-mod3"}</v>
+      </c>
+      <c r="P15" t="str">
+        <v>C:\Users\SO\Videos\intellectus\project-intellectus\storage\523221049457\GEOLOCALIZACIONES\10-02-2026,\523221049457_SO-POSITIVO.pdf</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>